<commit_message>
Added new RDF data schemes and visual schemes, fixed XLSX spreadsheets for economy-table50-54
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table51.xlsx
+++ b/sources/table_normalization/xlsx/economy-table51.xlsx
@@ -288,7 +288,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,7 +297,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -442,31 +448,31 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -891,16 +897,16 @@
   <sheetData>
     <row r="2" spans="1:5" ht="25.5" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" ht="25.5" customHeight="1">
       <c r="A3" s="2"/>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -913,7 +919,7 @@
     </row>
     <row r="4" spans="1:5" ht="25.5" customHeight="1">
       <c r="A4" s="2"/>
-      <c r="B4" s="13"/>
+      <c r="B4" s="7"/>
       <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
@@ -924,7 +930,7 @@
     </row>
     <row r="5" spans="1:5" ht="25.5" customHeight="1">
       <c r="A5" s="2"/>
-      <c r="B5" s="13"/>
+      <c r="B5" s="7"/>
       <c r="C5" s="4" t="s">
         <v>3</v>
       </c>
@@ -935,7 +941,7 @@
     </row>
     <row r="6" spans="1:5" ht="25.5" customHeight="1">
       <c r="A6" s="2"/>
-      <c r="B6" s="13"/>
+      <c r="B6" s="7"/>
       <c r="C6" s="4" t="s">
         <v>4</v>
       </c>
@@ -946,7 +952,7 @@
     </row>
     <row r="7" spans="1:5" ht="25.5" customHeight="1">
       <c r="A7" s="2"/>
-      <c r="B7" s="14"/>
+      <c r="B7" s="8"/>
       <c r="C7" s="4" t="s">
         <v>5</v>
       </c>
@@ -957,11 +963,11 @@
     </row>
     <row r="8" spans="1:5" ht="25.5" customHeight="1">
       <c r="A8" s="2"/>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8">
+      <c r="C8" s="11"/>
+      <c r="D8" s="9">
         <f>SUM(D3:D7)</f>
         <v>96172472</v>
       </c>
@@ -969,7 +975,7 @@
     </row>
     <row r="9" spans="1:5" ht="25.5" customHeight="1">
       <c r="A9" s="2"/>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="4" t="s">
@@ -982,7 +988,7 @@
     </row>
     <row r="10" spans="1:5" ht="25.5" customHeight="1">
       <c r="A10" s="2"/>
-      <c r="B10" s="13"/>
+      <c r="B10" s="7"/>
       <c r="C10" s="4" t="s">
         <v>2</v>
       </c>
@@ -993,7 +999,7 @@
     </row>
     <row r="11" spans="1:5" ht="25.5" customHeight="1">
       <c r="A11" s="2"/>
-      <c r="B11" s="13"/>
+      <c r="B11" s="7"/>
       <c r="C11" s="4" t="s">
         <v>3</v>
       </c>
@@ -1004,7 +1010,7 @@
     </row>
     <row r="12" spans="1:5" ht="25.5" customHeight="1">
       <c r="A12" s="2"/>
-      <c r="B12" s="13"/>
+      <c r="B12" s="7"/>
       <c r="C12" s="4" t="s">
         <v>4</v>
       </c>
@@ -1015,7 +1021,7 @@
     </row>
     <row r="13" spans="1:5" ht="25.5" customHeight="1">
       <c r="A13" s="2"/>
-      <c r="B13" s="14"/>
+      <c r="B13" s="8"/>
       <c r="C13" s="4" t="s">
         <v>5</v>
       </c>
@@ -1026,11 +1032,11 @@
     </row>
     <row r="14" spans="1:5" ht="25.5" customHeight="1">
       <c r="A14" s="2"/>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8">
+      <c r="C14" s="11"/>
+      <c r="D14" s="9">
         <f>SUM(D9:D13)</f>
         <v>101871312</v>
       </c>
@@ -1038,7 +1044,7 @@
     </row>
     <row r="15" spans="1:5" ht="25.5" customHeight="1">
       <c r="A15" s="2"/>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -1051,7 +1057,7 @@
     </row>
     <row r="16" spans="1:5" ht="25.5" customHeight="1">
       <c r="A16" s="2"/>
-      <c r="B16" s="13"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="4" t="s">
         <v>2</v>
       </c>
@@ -1062,7 +1068,7 @@
     </row>
     <row r="17" spans="1:5" ht="25.5" customHeight="1">
       <c r="A17" s="2"/>
-      <c r="B17" s="13"/>
+      <c r="B17" s="7"/>
       <c r="C17" s="4" t="s">
         <v>3</v>
       </c>
@@ -1073,7 +1079,7 @@
     </row>
     <row r="18" spans="1:5" ht="25.5" customHeight="1">
       <c r="A18" s="2"/>
-      <c r="B18" s="13"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="4" t="s">
         <v>4</v>
       </c>
@@ -1084,7 +1090,7 @@
     </row>
     <row r="19" spans="1:5" ht="25.5" customHeight="1">
       <c r="A19" s="2"/>
-      <c r="B19" s="14"/>
+      <c r="B19" s="8"/>
       <c r="C19" s="4" t="s">
         <v>5</v>
       </c>
@@ -1095,11 +1101,11 @@
     </row>
     <row r="20" spans="1:5" ht="25.5" customHeight="1">
       <c r="A20" s="2"/>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="8">
+      <c r="C20" s="13"/>
+      <c r="D20" s="9">
         <f>SUM(D15:D19)</f>
         <v>4947402</v>
       </c>

</xml_diff>